<commit_message>
Agrega URLs de imagen reales para 35 viviendas
Se cargaron por ID (sin tocar filas ni columnas existentes) las URLs
de foto que el usuario obtuvo de Inmuebles24, incluyendo las primeras
5 propiedades del catalogo. Quedan pendientes las 6 propiedades cuyas
URLs no vinieron en el archivo subido (IDs 8, 15, 16, 30, 32, 34).
</commit_message>
<xml_diff>
--- a/Viviendas_en_Venta_La_Paz.xlsx
+++ b/Viviendas_en_Venta_La_Paz.xlsx
@@ -753,7 +753,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P2" s="19" t="n"/>
+      <c r="P2" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/48/92/61/90/1200x1200/1587104686.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="25.5" customHeight="1" s="9">
       <c r="A3" s="2" t="n">
@@ -814,7 +818,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P3" s="19" t="n"/>
+      <c r="P3" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/10/76/67/1200x1200/1590644718.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="25.5" customHeight="1" s="9">
       <c r="A4" s="2" t="n">
@@ -875,7 +883,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P4" s="19" t="n"/>
+      <c r="P4" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/74/11/45/1200x1200/1603847351.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="25.5" customHeight="1" s="9">
       <c r="A5" s="2" t="n">
@@ -936,7 +948,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P5" s="19" t="n"/>
+      <c r="P5" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/50/67/61/67/1200x1200/1623184900.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="25.5" customHeight="1" s="9">
       <c r="A6" s="2" t="n">
@@ -997,7 +1013,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P6" s="19" t="n"/>
+      <c r="P6" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/65/28/67/1200x1200/1602057090.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="25.5" customHeight="1" s="9">
       <c r="A7" s="2" t="n">
@@ -1062,7 +1082,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P7" s="19" t="n"/>
+      <c r="P7" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/65/53/09/1200x1200/1602106805.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="25.5" customHeight="1" s="9">
       <c r="A8" s="2" t="n">
@@ -1123,7 +1147,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P8" s="19" t="n"/>
+      <c r="P8" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/18/01/49/52/07/75/360x266/1599173160.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="25.5" customHeight="1" s="9">
       <c r="A9" s="2" t="n">
@@ -1253,7 +1281,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P10" s="19" t="n"/>
+      <c r="P10" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/57/92/31/1200x1200/1600490803.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="38.25" customHeight="1" s="9">
       <c r="A11" s="2" t="n">
@@ -1318,7 +1350,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P11" s="19" t="n"/>
+      <c r="P11" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/50/11/21/02/1200x1200/1611411915.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="25.5" customHeight="1" s="9">
       <c r="A12" s="2" t="n">
@@ -1379,7 +1415,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P12" s="19" t="n"/>
+      <c r="P12" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/20/41/93/1200x1200/1592569753.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" s="9">
       <c r="A13" s="2" t="n">
@@ -1440,7 +1480,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P13" s="19" t="n"/>
+      <c r="P13" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/45/46/72/21/1200x1200/1504957360.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="25.5" customHeight="1" s="9">
       <c r="A14" s="2" t="n">
@@ -1505,7 +1549,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P14" s="19" t="n"/>
+      <c r="P14" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/00/91/10/54/16/1200x1200/1114614444.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="25.5" customHeight="1" s="9">
       <c r="A15" s="2" t="n">
@@ -1566,7 +1614,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P15" s="19" t="n"/>
+      <c r="P15" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/60/70/64/1200x1200/1621653553.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="25.5" customHeight="1" s="9">
       <c r="A16" s="2" t="n">
@@ -1753,7 +1805,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P18" s="19" t="n"/>
+      <c r="P18" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/64/65/02/1200x1200/1601934402.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="25.5" customHeight="1" s="9">
       <c r="A19" s="2" t="n">
@@ -1814,7 +1870,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P19" s="19" t="n"/>
+      <c r="P19" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/46/80/92/11/1200x1200/1586532946.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="25.5" customHeight="1" s="9">
       <c r="A20" s="2" t="n">
@@ -1875,7 +1935,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P20" s="19" t="n"/>
+      <c r="P20" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/50/24/55/38/1200x1200/1614080409.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="25.5" customHeight="1" s="9">
       <c r="A21" s="2" t="n">
@@ -1940,7 +2004,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P21" s="19" t="n"/>
+      <c r="P21" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/48/20/12/18/1200x1200/1601440423.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="25.5" customHeight="1" s="9">
       <c r="A22" s="2" t="n">
@@ -2001,7 +2069,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P22" s="19" t="n"/>
+      <c r="P22" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/48/19/18/21/1200x1200/1601444774.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="25.5" customHeight="1" s="9">
       <c r="A23" s="2" t="n">
@@ -2062,7 +2134,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P23" s="19" t="n"/>
+      <c r="P23" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/45/27/42/86/1200x1200/1624853443.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="25.5" customHeight="1" s="9">
       <c r="A24" s="2" t="n">
@@ -2123,7 +2199,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P24" s="19" t="n"/>
+      <c r="P24" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/46/61/53/66/1200x1200/1578338508.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="25.5" customHeight="1" s="9">
       <c r="A25" s="2" t="n">
@@ -2180,7 +2260,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P25" s="19" t="n"/>
+      <c r="P25" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/48/98/33/90/1200x1200/1588238517.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="25.5" customHeight="1" s="9">
       <c r="A26" s="2" t="n">
@@ -2241,7 +2325,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P26" s="19" t="n"/>
+      <c r="P26" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/46/26/84/79/1200x1200/1590095756.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="25.5" customHeight="1" s="9">
       <c r="A27" s="2" t="n">
@@ -2302,7 +2390,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P27" s="19" t="n"/>
+      <c r="P27" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/45/22/98/98/1200x1200/1561323415.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="25.5" customHeight="1" s="9">
       <c r="A28" s="2" t="n">
@@ -2363,7 +2455,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P28" s="19" t="n"/>
+      <c r="P28" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/18/01/50/51/18/37/360x266/1619879156.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="25.5" customHeight="1" s="9">
       <c r="A29" s="2" t="n">
@@ -2424,7 +2520,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P29" s="19" t="n"/>
+      <c r="P29" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/50/62/78/21/1200x1200/1622151517.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="25.5" customHeight="1" s="9">
       <c r="A30" s="2" t="n">
@@ -2485,7 +2585,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P30" s="19" t="n"/>
+      <c r="P30" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/38/29/29/1200x1200/1596302391.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="25.5" customHeight="1" s="9">
       <c r="A31" s="2" t="n">
@@ -2607,7 +2711,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P32" s="19" t="n"/>
+      <c r="P32" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/49/32/53/03/1200x1200/1595139090.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="25.5" customHeight="1" s="9">
       <c r="A33" s="2" t="n">
@@ -2729,7 +2837,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P34" s="19" t="n"/>
+      <c r="P34" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/48/77/63/81/1200x1200/1584238159.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="25.5" customHeight="1" s="9">
       <c r="A35" s="2" t="n">
@@ -2851,7 +2963,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P36" s="19" t="n"/>
+      <c r="P36" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/46/26/99/01/1200x1200/1527813686.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="25.5" customHeight="1" s="9">
       <c r="A37" s="2" t="n">
@@ -2912,7 +3028,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P37" s="19" t="n"/>
+      <c r="P37" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/47/44/77/51/1200x1200/1556642759.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="25.5" customHeight="1" s="9">
       <c r="A38" s="2" t="n">
@@ -2973,7 +3093,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P38" s="19" t="n"/>
+      <c r="P38" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/18/01/48/70/21/44/360x266/1582831439.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="25.5" customHeight="1" s="9">
       <c r="A39" s="2" t="n">
@@ -3034,7 +3158,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P39" s="19" t="n"/>
+      <c r="P39" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/47/44/77/51/1200x1200/1556642759.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="25.5" customHeight="1" s="9">
       <c r="A40" s="2" t="n">
@@ -3095,7 +3223,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P40" s="19" t="n"/>
+      <c r="P40" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/46/78/57/70/1200x1200/1540402288.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="25.5" customHeight="1" s="9">
       <c r="A41" s="2" t="n">
@@ -3156,7 +3288,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P41" s="19" t="n"/>
+      <c r="P41" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/resize/18/01/50/62/43/55/1200x1200/1622077922.jpg?isFirstImage=true</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="25.5" customHeight="1" s="9">
       <c r="A42" s="2" t="n">
@@ -3221,7 +3357,11 @@
           <t>Ver listado</t>
         </is>
       </c>
-      <c r="P42" s="19" t="n"/>
+      <c r="P42" s="19" t="inlineStr">
+        <is>
+          <t>https://img10.naventcdn.com/avisos/18/01/50/54/56/94/360x266/1620529487.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="25.5" customHeight="1" s="9">
       <c r="A43" s="2" t="n">

</xml_diff>